<commit_message>
CalculatedAADT: fill the template in LibreOffice so the leg sketch and header survive
make_calculated_aadt.py now opens the original .xls template headless via
Python UNO, writes the study inputs, and stores the .xls and .xlsx from
that document: the drawn intersection lines, the two-line page header
and the superscript footnote markers are kept, short template-style leg
names fit the cells, notes wrap within the sheet, and the 4-LEG sheet
prints on one page. Values unchanged (total 12,050, 2.03 %, keep 12,300).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012AMZ23B9M2AjrQa7UP3LHH
</commit_message>
<xml_diff>
--- a/HSIP/41000079736/41000079736_CalculatedAADT.xlsx
+++ b/HSIP/41000079736/41000079736_CalculatedAADT.xlsx
@@ -262,8 +262,10 @@
   <si>
     <r>
       <rPr>
+        <i val="true"/>
         <vertAlign val="superscript"/>
         <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
       </rPr>
@@ -271,7 +273,9 @@
     </r>
     <r>
       <rPr>
+        <i val="true"/>
         <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
       </rPr>
@@ -279,22 +283,104 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">   (1,300) NCDOT counts, rounded per the NCDOT/AASHTO AADT rounding chart (nearest 100 for 1,000-9,999).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   The other legs are the published 2021 NCDOT counts. Legs: N/S = NC 180/NC 226 (S Post Rd), stations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   0230000187 (N) and 0230000152 (S); NW = SR 1103 (Pleasant Dr), station 0230000045; SE = SR 1103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   (Pleasant Hill Church Rd), station 0230000531.</t>
-  </si>
-  <si>
     <r>
       <rPr>
+        <i val="true"/>
         <vertAlign val="superscript"/>
         <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">(1,300) NCDOT counts, rounded per the NCDOT/AASHTO AADT rounding chart (nearest 100 for 1,000-9,999).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">The other legs are the published 2021 NCDOT counts. Legs: N/S = NC 180/NC 226 (S Post Rd), stations</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">0230000187 (N) and 0230000152 (S); NW = SR 1103 (Pleasant Dr), station 0230000045; SE = SR 1103</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">(Pleasant Hill Church Rd), station 0230000531.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="true"/>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
       </rPr>
@@ -302,7 +388,9 @@
     </r>
     <r>
       <rPr>
+        <i val="true"/>
         <sz val="10"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
       </rPr>
@@ -668,7 +756,7 @@
     <numFmt numFmtId="172" formatCode="[$-409]m/d/yyyy"/>
     <numFmt numFmtId="173" formatCode="0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -757,8 +845,17 @@
       <family val="2"/>
     </font>
     <font>
+      <i val="true"/>
       <vertAlign val="superscript"/>
       <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
     </font>
@@ -1092,7 +1189,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1100,11 +1197,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3850,7 +3947,7 @@
       <c r="G49" s="3"/>
     </row>
     <row r="50" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="56" t="s">
         <v>41</v>
       </c>
       <c r="B50" s="3"/>
@@ -3861,7 +3958,7 @@
       <c r="G50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="56" t="s">
         <v>42</v>
       </c>
       <c r="B51" s="3"/>
@@ -3872,7 +3969,7 @@
       <c r="G51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="56" t="s">
         <v>43</v>
       </c>
       <c r="B52" s="3"/>
@@ -3883,7 +3980,7 @@
       <c r="G52" s="3"/>
     </row>
     <row r="53" customFormat="false" ht="13.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="56" t="s">
         <v>44</v>
       </c>
       <c r="B53" s="3"/>

</xml_diff>